<commit_message>
new datasheets for EA/XRF (Aug 2026)
</commit_message>
<xml_diff>
--- a/Jordan Leaf and Compost Sample Sheet 2024-2025.xlsx
+++ b/Jordan Leaf and Compost Sample Sheet 2024-2025.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ellieandrews/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zhang\Documents\GitHub\Andrews_CompostMulch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4E3637C-7C85-AC46-B94A-0D352657E0EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D523E65-C128-4AB2-99C5-CF53414E6C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24860" yWindow="4200" windowWidth="26340" windowHeight="22840" xr2:uid="{815BCD88-345A-3D48-A8DA-118F945F21B4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{815BCD88-345A-3D48-A8DA-118F945F21B4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Feb_2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Aug_2026" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="32">
   <si>
     <t>Sample</t>
   </si>
@@ -490,16 +491,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E98FB7BB-CC74-2442-9AF5-1CABEBD695BF}">
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.1640625" customWidth="1"/>
+    <col min="1" max="1" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.125" customWidth="1"/>
     <col min="3" max="3" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -558,7 +559,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -575,7 +576,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -592,7 +593,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -609,7 +610,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -626,7 +627,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -643,7 +644,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -660,7 +661,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -677,7 +678,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -694,7 +695,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -711,7 +712,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -728,7 +729,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -745,7 +746,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -762,7 +763,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -779,7 +780,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -796,7 +797,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -813,7 +814,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -830,7 +831,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -847,7 +848,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -864,7 +865,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -881,7 +882,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -898,7 +899,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -915,7 +916,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -932,7 +933,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -949,7 +950,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -966,7 +967,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -983,7 +984,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1000,7 +1001,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1017,7 +1018,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1034,7 +1035,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1051,7 +1052,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1068,7 +1069,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1085,7 +1086,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1102,7 +1103,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1119,7 +1120,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1136,7 +1137,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1153,7 +1154,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1170,7 +1171,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1187,7 +1188,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1204,7 +1205,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1221,7 +1222,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1238,7 +1239,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1255,7 +1256,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1272,7 +1273,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1289,7 +1290,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1306,7 +1307,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1323,7 +1324,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1340,7 +1341,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1357,7 +1358,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1374,7 +1375,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1385,7 +1386,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1396,7 +1397,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1407,7 +1408,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1418,7 +1419,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1429,7 +1430,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1440,7 +1441,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1451,7 +1452,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1462,7 +1463,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1473,7 +1474,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -1484,7 +1485,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -1499,4 +1500,162 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1F001CB-FCE1-4872-9934-6B74DC3151FF}">
+  <dimension ref="A1:A29"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>